<commit_message>
new file Quantitative Form Responses
</commit_message>
<xml_diff>
--- a/Data/Quantitative Form Responses.xlsx
+++ b/Data/Quantitative Form Responses.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Respostas ao formulário 1" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Results" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -161,7 +161,7 @@
     <t>De acordo</t>
   </si>
   <si>
-    <t>Carlos Andrew Costa Bezerra</t>
+    <t>Participant 1</t>
   </si>
   <si>
     <t>APIs</t>
@@ -179,7 +179,7 @@
     <t>1 - Não</t>
   </si>
   <si>
-    <t>Túlio Bezerra Machado</t>
+    <t>Participant 2</t>
   </si>
   <si>
     <t>Aplicações Mobile</t>
@@ -188,337 +188,337 @@
     <t>5 - Totalmente</t>
   </si>
   <si>
-    <t>Weberson Ribeiro Santana</t>
-  </si>
-  <si>
-    <t>EMERSON MARTINS DA SILVA</t>
+    <t>Participant 3</t>
+  </si>
+  <si>
+    <t>Participant 4</t>
   </si>
   <si>
     <t>Web</t>
   </si>
   <si>
-    <t xml:space="preserve">Junior Vinicius Silva </t>
-  </si>
-  <si>
-    <t>Thiago Victor Fragoso Guimarães Bello</t>
+    <t>Participant 5</t>
+  </si>
+  <si>
+    <t>Participant 6</t>
   </si>
   <si>
     <t>IA</t>
   </si>
   <si>
-    <t>Rendrikson de Oliveira Soares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">José Ferreira Leite Neto </t>
-  </si>
-  <si>
-    <t>Katiano  Marcio da Silva</t>
+    <t>Participant 7</t>
+  </si>
+  <si>
+    <t>Participant 8</t>
+  </si>
+  <si>
+    <t>Participant 9</t>
   </si>
   <si>
     <t>Plataforma em Nuvem</t>
   </si>
   <si>
-    <t xml:space="preserve">Claudeci Siqueira de Lucena Júnior </t>
-  </si>
-  <si>
-    <t>Everson Vinicius Soares do Nascimento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cláudio J R Cavalcanti </t>
-  </si>
-  <si>
-    <t>Eliton Freitas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlos Augusto Pereira Barbosa </t>
-  </si>
-  <si>
-    <t>Juliano Araújo Farias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Larissa Marinho </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rafael Fernandes Pugliese de Morais </t>
-  </si>
-  <si>
-    <t>Andressa Carvalho Melo da Silveira</t>
-  </si>
-  <si>
-    <t>Emerson Paulo Soares de Souza</t>
-  </si>
-  <si>
-    <t>Diogo Vieira Buíque</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adinã Genaro </t>
-  </si>
-  <si>
-    <t>Manuele Ferreira</t>
+    <t>Participant 10</t>
+  </si>
+  <si>
+    <t>Participant 11</t>
+  </si>
+  <si>
+    <t>Participant 12</t>
+  </si>
+  <si>
+    <t>Participant 13</t>
+  </si>
+  <si>
+    <t>Participant 14</t>
+  </si>
+  <si>
+    <t>Participant 15</t>
+  </si>
+  <si>
+    <t>Participant 16</t>
+  </si>
+  <si>
+    <t>Participant 17</t>
+  </si>
+  <si>
+    <t>Participant 18</t>
+  </si>
+  <si>
+    <t>Participant 19</t>
+  </si>
+  <si>
+    <t>Participant 20</t>
+  </si>
+  <si>
+    <t>Participant 21</t>
+  </si>
+  <si>
+    <t>Participant 22</t>
   </si>
   <si>
     <t>Dados</t>
   </si>
   <si>
-    <t xml:space="preserve">Henrique Passine Moreira </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reinaldo </t>
+    <t>Participant 23</t>
+  </si>
+  <si>
+    <t>Participant 24</t>
   </si>
   <si>
     <t>Desktop</t>
   </si>
   <si>
-    <t>Reginaldo Ramos</t>
-  </si>
-  <si>
-    <t>Roberta Silva Delbany</t>
-  </si>
-  <si>
-    <t>Erica Acioli</t>
-  </si>
-  <si>
-    <t>Doug Caval Korsonovitch</t>
-  </si>
-  <si>
-    <t>André Felipe Mota Belforte</t>
-  </si>
-  <si>
-    <t>Rachel Teixeira Chicanelli</t>
-  </si>
-  <si>
-    <t>Gabriel Campos Pereira dos Santos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isna Nogueira Faria </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ligia Barbosa Menezes </t>
-  </si>
-  <si>
-    <t>Arnaldo Nogueira Paraguassú</t>
-  </si>
-  <si>
-    <t>Fabiano Ortis</t>
-  </si>
-  <si>
-    <t>Ricardo Augusto de Moura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michellen Gabriel </t>
+    <t>Participant 25</t>
+  </si>
+  <si>
+    <t>Participant 26</t>
+  </si>
+  <si>
+    <t>Participant 27</t>
+  </si>
+  <si>
+    <t>Participant 28</t>
+  </si>
+  <si>
+    <t>Participant 29</t>
+  </si>
+  <si>
+    <t>Participant 30</t>
+  </si>
+  <si>
+    <t>Participant 31</t>
+  </si>
+  <si>
+    <t>Participant 32</t>
+  </si>
+  <si>
+    <t>Participant 33</t>
+  </si>
+  <si>
+    <t>Participant 34</t>
+  </si>
+  <si>
+    <t>Participant 35</t>
+  </si>
+  <si>
+    <t>Participant 36</t>
+  </si>
+  <si>
+    <t>Participant 37</t>
   </si>
   <si>
     <t>Sistemas Embarcados</t>
   </si>
   <si>
-    <t>Alessandra H, igrissis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sheila Barreto </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gesane Caroline </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patricia Maroubo </t>
-  </si>
-  <si>
-    <t>M. Cristina Zanutto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heloar Cristina Alves da Silva </t>
+    <t>Participant 38</t>
+  </si>
+  <si>
+    <t>Participant 39</t>
+  </si>
+  <si>
+    <t>Participant 40</t>
+  </si>
+  <si>
+    <t>Participant 41</t>
+  </si>
+  <si>
+    <t>Participant 42</t>
+  </si>
+  <si>
+    <t>Participant 43</t>
   </si>
   <si>
     <t xml:space="preserve">Inteligência Artificial </t>
   </si>
   <si>
-    <t>Kevin Tenório Lobo Martins de Souza</t>
-  </si>
-  <si>
-    <t>Gabriel de Carvalho Freitas</t>
-  </si>
-  <si>
-    <t>Douglas Chalegre De Sá Belo Torres</t>
-  </si>
-  <si>
-    <t>Mauri Goncalves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michele Daniele da Silva Aguiar Barbosa </t>
-  </si>
-  <si>
-    <t>Kimbi jabez bongi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natalia Carvalho Molina </t>
-  </si>
-  <si>
-    <t>Guilherme Oliveira Vaz</t>
-  </si>
-  <si>
-    <t>Rodrigo Romero Costa da Matta Monteiro</t>
-  </si>
-  <si>
-    <t>Andrea Rodrigues</t>
-  </si>
-  <si>
-    <t>Fernando Calixto de Oliveira Tenório</t>
-  </si>
-  <si>
-    <t>Jorge Chaffin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Larissa da Silva Santos </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liedson Danubio Oliveira Leite </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yuri Santos de Farias </t>
-  </si>
-  <si>
-    <t>Sonia silva</t>
-  </si>
-  <si>
-    <t>Vanessa Ferreira Tornich</t>
-  </si>
-  <si>
-    <t>Ivan Monma</t>
-  </si>
-  <si>
-    <t>Wanderley Graça Rivela Junior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Máyra Garcia Alves </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Talita Assis Silva de Jesus </t>
-  </si>
-  <si>
-    <t>Jessica Mitui de Goes</t>
-  </si>
-  <si>
-    <t>Bárbara Nascimento Candido de Oliveira</t>
-  </si>
-  <si>
-    <t>Matheus Rezende Pereira</t>
-  </si>
-  <si>
-    <t>Fernando Gouveia</t>
-  </si>
-  <si>
-    <t>William Pereira Terra</t>
-  </si>
-  <si>
-    <t>Hugo Hoffmann</t>
+    <t>Participant 44</t>
+  </si>
+  <si>
+    <t>Participant 45</t>
+  </si>
+  <si>
+    <t>Participant 46</t>
+  </si>
+  <si>
+    <t>Participant 47</t>
+  </si>
+  <si>
+    <t>Participant 48</t>
+  </si>
+  <si>
+    <t>Participant 49</t>
+  </si>
+  <si>
+    <t>Participant 50</t>
+  </si>
+  <si>
+    <t>Participant 51</t>
+  </si>
+  <si>
+    <t>Participant 52</t>
+  </si>
+  <si>
+    <t>Participant 53</t>
+  </si>
+  <si>
+    <t>Participant 54</t>
+  </si>
+  <si>
+    <t>Participant 55</t>
+  </si>
+  <si>
+    <t>Participant 56</t>
+  </si>
+  <si>
+    <t>Participant 57</t>
+  </si>
+  <si>
+    <t>Participant 58</t>
+  </si>
+  <si>
+    <t>Participant 59</t>
+  </si>
+  <si>
+    <t>Participant 60</t>
+  </si>
+  <si>
+    <t>Participant 61</t>
+  </si>
+  <si>
+    <t>Participant 62</t>
+  </si>
+  <si>
+    <t>Participant 63</t>
+  </si>
+  <si>
+    <t>Participant 64</t>
+  </si>
+  <si>
+    <t>Participant 65</t>
+  </si>
+  <si>
+    <t>Participant 66</t>
+  </si>
+  <si>
+    <t>Participant 67</t>
+  </si>
+  <si>
+    <t>Participant 68</t>
+  </si>
+  <si>
+    <t>Participant 69</t>
+  </si>
+  <si>
+    <t>Participant 70</t>
   </si>
   <si>
     <t>IoT</t>
   </si>
   <si>
-    <t>Karoline Cianci Gishitomi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Roberto Trintin </t>
-  </si>
-  <si>
-    <t>vanessa do nascimento</t>
-  </si>
-  <si>
-    <t>Flaviano José de Lima Viana</t>
-  </si>
-  <si>
-    <t>Rômulo Crestan Gomes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gilza Plaques de Souza </t>
-  </si>
-  <si>
-    <t>Thássio Costa de Oliveira Anselmo</t>
+    <t>Participant 71</t>
+  </si>
+  <si>
+    <t>Participant 72</t>
+  </si>
+  <si>
+    <t>Participant 73</t>
+  </si>
+  <si>
+    <t>Participant 74</t>
+  </si>
+  <si>
+    <t>Participant 75</t>
+  </si>
+  <si>
+    <t>Participant 76</t>
+  </si>
+  <si>
+    <t>Participant 77</t>
   </si>
   <si>
     <t>Aplicações bancárias</t>
   </si>
   <si>
-    <t xml:space="preserve">Afonso de Jesus Pimentel Alves </t>
+    <t>Participant 78</t>
   </si>
   <si>
     <t>CRM com IA embarcada</t>
   </si>
   <si>
-    <t>Beatriz Ereno</t>
-  </si>
-  <si>
-    <t>Victória Borges</t>
-  </si>
-  <si>
-    <t>TADEU PEREIRA DOS SANTOS</t>
-  </si>
-  <si>
-    <t>Raul Alves de Almeida</t>
-  </si>
-  <si>
-    <t>Margarete Alves Andrade</t>
+    <t>Participant 79</t>
+  </si>
+  <si>
+    <t>Participant 80</t>
+  </si>
+  <si>
+    <t>Participant 81</t>
+  </si>
+  <si>
+    <t>Participant 82</t>
+  </si>
+  <si>
+    <t>Participant 83</t>
   </si>
   <si>
     <t>Plataforma Digital</t>
   </si>
   <si>
-    <t xml:space="preserve">Diego Henrique Rodrigues Pereira </t>
-  </si>
-  <si>
-    <t>Carlos Hung</t>
-  </si>
-  <si>
-    <t>Marcela Spindola de Oliveira</t>
-  </si>
-  <si>
-    <t>Daniel Costa de Faria</t>
-  </si>
-  <si>
-    <t>Sandra Machado da Costa</t>
-  </si>
-  <si>
-    <t>Darlan Dalsasso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raissa Pires Camelo Schindler </t>
-  </si>
-  <si>
-    <t>Tamara Lima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maria Aparecida Ignacio Cavanha Nascimento </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gislene da Anunciação Oliveira </t>
-  </si>
-  <si>
-    <t>Luisa jazyk</t>
-  </si>
-  <si>
-    <t>Thiago Carneiro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guilherme Ventura dos Santos </t>
-  </si>
-  <si>
-    <t>Amanda Cristina Ferreira Nazaretto</t>
-  </si>
-  <si>
-    <t>Felipe Calasans de Sousa</t>
-  </si>
-  <si>
-    <t>Cendy Mara dos Santos Cabral</t>
-  </si>
-  <si>
-    <t>Raquel Falcão l</t>
-  </si>
-  <si>
-    <t>Francisco Assis Saraiva de Oliveira</t>
-  </si>
-  <si>
-    <t>Diego Nunes</t>
+    <t>Participant 84</t>
+  </si>
+  <si>
+    <t>Participant 85</t>
+  </si>
+  <si>
+    <t>Participant 86</t>
+  </si>
+  <si>
+    <t>Participant 87</t>
+  </si>
+  <si>
+    <t>Participant 88</t>
+  </si>
+  <si>
+    <t>Participant 89</t>
+  </si>
+  <si>
+    <t>Participant 90</t>
+  </si>
+  <si>
+    <t>Participant 91</t>
+  </si>
+  <si>
+    <t>Participant 92</t>
+  </si>
+  <si>
+    <t>Participant 93</t>
+  </si>
+  <si>
+    <t>Participant 94</t>
+  </si>
+  <si>
+    <t>Participant 95</t>
+  </si>
+  <si>
+    <t>Participant 96</t>
+  </si>
+  <si>
+    <t>Participant 97</t>
+  </si>
+  <si>
+    <t>Participant 98</t>
+  </si>
+  <si>
+    <t>Participant 99</t>
+  </si>
+  <si>
+    <t>Participant 100</t>
+  </si>
+  <si>
+    <t>Participant 101</t>
+  </si>
+  <si>
+    <t>Participant 102</t>
   </si>
 </sst>
 </file>
@@ -559,7 +559,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -574,6 +574,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,7 +622,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="3" pivot="0" name="Respostas ao formulário 1-style">
+    <tableStyle count="3" pivot="0" name="Results-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -676,7 +679,7 @@
     <tableColumn name="35 - O consumo energético é monitorado com o mesmo rigor que desempenho e segurança?" id="39"/>
     <tableColumn name="Coluna 39" id="40"/>
   </tableColumns>
-  <tableStyleInfo name="Respostas ao formulário 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Results-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -1018,7 +1021,7 @@
       <c r="B2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>41</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -1138,7 +1141,7 @@
       <c r="B3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>47</v>
       </c>
       <c r="D3" s="4" t="s">
@@ -1258,7 +1261,7 @@
       <c r="B4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>50</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -1378,7 +1381,7 @@
       <c r="B5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D5" s="4" t="s">
@@ -1498,7 +1501,7 @@
       <c r="B6" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>53</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -1618,7 +1621,7 @@
       <c r="B7" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="4" t="s">
@@ -1738,7 +1741,7 @@
       <c r="B8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>56</v>
       </c>
       <c r="D8" s="4" t="s">
@@ -1858,7 +1861,7 @@
       <c r="B9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -1978,7 +1981,7 @@
       <c r="B10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>58</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -2098,7 +2101,7 @@
       <c r="B11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>60</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -2218,7 +2221,7 @@
       <c r="B12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D12" s="4" t="s">
@@ -2338,7 +2341,7 @@
       <c r="B13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -2458,7 +2461,7 @@
       <c r="B14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>63</v>
       </c>
       <c r="D14" s="4" t="s">
@@ -2578,7 +2581,7 @@
       <c r="B15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>64</v>
       </c>
       <c r="D15" s="4" t="s">
@@ -2698,7 +2701,7 @@
       <c r="B16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>65</v>
       </c>
       <c r="D16" s="4" t="s">
@@ -2818,7 +2821,7 @@
       <c r="B17" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>66</v>
       </c>
       <c r="D17" s="4" t="s">
@@ -2938,7 +2941,7 @@
       <c r="B18" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>67</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -3058,7 +3061,7 @@
       <c r="B19" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>68</v>
       </c>
       <c r="D19" s="4" t="s">
@@ -3178,7 +3181,7 @@
       <c r="B20" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D20" s="4" t="s">
@@ -3298,7 +3301,7 @@
       <c r="B21" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>70</v>
       </c>
       <c r="D21" s="4" t="s">
@@ -3418,7 +3421,7 @@
       <c r="B22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -3538,7 +3541,7 @@
       <c r="B23" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>72</v>
       </c>
       <c r="D23" s="4" t="s">
@@ -3658,7 +3661,7 @@
       <c r="B24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>74</v>
       </c>
       <c r="D24" s="4" t="s">
@@ -3778,7 +3781,7 @@
       <c r="B25" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="5" t="s">
         <v>75</v>
       </c>
       <c r="D25" s="4" t="s">
@@ -3898,7 +3901,7 @@
       <c r="B26" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>77</v>
       </c>
       <c r="D26" s="4" t="s">
@@ -4018,7 +4021,7 @@
       <c r="B27" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="5" t="s">
         <v>78</v>
       </c>
       <c r="D27" s="4" t="s">
@@ -4138,7 +4141,7 @@
       <c r="B28" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>79</v>
       </c>
       <c r="D28" s="4" t="s">
@@ -4258,7 +4261,7 @@
       <c r="B29" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="5" t="s">
         <v>80</v>
       </c>
       <c r="D29" s="4" t="s">
@@ -4378,7 +4381,7 @@
       <c r="B30" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="5" t="s">
         <v>81</v>
       </c>
       <c r="D30" s="4" t="s">
@@ -4498,7 +4501,7 @@
       <c r="B31" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="5" t="s">
         <v>82</v>
       </c>
       <c r="D31" s="4" t="s">
@@ -4618,7 +4621,7 @@
       <c r="B32" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D32" s="4" t="s">
@@ -4738,7 +4741,7 @@
       <c r="B33" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="5" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="4" t="s">
@@ -4858,7 +4861,7 @@
       <c r="B34" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D34" s="4" t="s">
@@ -4978,7 +4981,7 @@
       <c r="B35" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="5" t="s">
         <v>86</v>
       </c>
       <c r="D35" s="4" t="s">
@@ -5098,7 +5101,7 @@
       <c r="B36" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="5" t="s">
         <v>87</v>
       </c>
       <c r="D36" s="4" t="s">
@@ -5218,7 +5221,7 @@
       <c r="B37" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="5" t="s">
         <v>88</v>
       </c>
       <c r="D37" s="4" t="s">
@@ -5338,7 +5341,7 @@
       <c r="B38" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="5" t="s">
         <v>89</v>
       </c>
       <c r="D38" s="4" t="s">
@@ -5458,7 +5461,7 @@
       <c r="B39" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="5" t="s">
         <v>91</v>
       </c>
       <c r="D39" s="4" t="s">
@@ -5578,7 +5581,7 @@
       <c r="B40" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="5" t="s">
         <v>92</v>
       </c>
       <c r="D40" s="4" t="s">
@@ -5698,7 +5701,7 @@
       <c r="B41" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="5" t="s">
         <v>93</v>
       </c>
       <c r="D41" s="4" t="s">
@@ -5818,7 +5821,7 @@
       <c r="B42" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="5" t="s">
         <v>94</v>
       </c>
       <c r="D42" s="4" t="s">
@@ -5938,7 +5941,7 @@
       <c r="B43" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="5" t="s">
         <v>95</v>
       </c>
       <c r="D43" s="4" t="s">
@@ -6058,7 +6061,7 @@
       <c r="B44" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="5" t="s">
         <v>96</v>
       </c>
       <c r="D44" s="4" t="s">
@@ -6178,7 +6181,7 @@
       <c r="B45" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="5" t="s">
         <v>98</v>
       </c>
       <c r="D45" s="4" t="s">
@@ -6298,7 +6301,7 @@
       <c r="B46" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="5" t="s">
         <v>99</v>
       </c>
       <c r="D46" s="4" t="s">
@@ -6418,7 +6421,7 @@
       <c r="B47" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="5" t="s">
         <v>100</v>
       </c>
       <c r="D47" s="4" t="s">
@@ -6538,7 +6541,7 @@
       <c r="B48" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="5" t="s">
         <v>101</v>
       </c>
       <c r="D48" s="4" t="s">
@@ -6658,7 +6661,7 @@
       <c r="B49" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D49" s="4" t="s">
@@ -6778,7 +6781,7 @@
       <c r="B50" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="5" t="s">
         <v>103</v>
       </c>
       <c r="D50" s="4" t="s">
@@ -6898,7 +6901,7 @@
       <c r="B51" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="5" t="s">
         <v>104</v>
       </c>
       <c r="D51" s="4" t="s">
@@ -7018,7 +7021,7 @@
       <c r="B52" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="5" t="s">
         <v>105</v>
       </c>
       <c r="D52" s="4" t="s">
@@ -7138,7 +7141,7 @@
       <c r="B53" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="5" t="s">
         <v>106</v>
       </c>
       <c r="D53" s="4" t="s">
@@ -7258,7 +7261,7 @@
       <c r="B54" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C54" s="5" t="s">
         <v>107</v>
       </c>
       <c r="D54" s="4" t="s">
@@ -7378,7 +7381,7 @@
       <c r="B55" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="5" t="s">
         <v>108</v>
       </c>
       <c r="D55" s="4" t="s">
@@ -7498,7 +7501,7 @@
       <c r="B56" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="5" t="s">
         <v>109</v>
       </c>
       <c r="D56" s="4" t="s">
@@ -7618,7 +7621,7 @@
       <c r="B57" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C57" s="5" t="s">
         <v>110</v>
       </c>
       <c r="D57" s="4" t="s">
@@ -7738,7 +7741,7 @@
       <c r="B58" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="C58" s="5" t="s">
         <v>111</v>
       </c>
       <c r="D58" s="4" t="s">
@@ -7858,7 +7861,7 @@
       <c r="B59" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="5" t="s">
         <v>112</v>
       </c>
       <c r="D59" s="4" t="s">
@@ -7978,7 +7981,7 @@
       <c r="B60" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="5" t="s">
         <v>113</v>
       </c>
       <c r="D60" s="4" t="s">
@@ -8098,7 +8101,7 @@
       <c r="B61" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="5" t="s">
         <v>114</v>
       </c>
       <c r="D61" s="4" t="s">
@@ -8218,7 +8221,7 @@
       <c r="B62" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="C62" s="5" t="s">
         <v>115</v>
       </c>
       <c r="D62" s="4" t="s">
@@ -8338,7 +8341,7 @@
       <c r="B63" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C63" s="4" t="s">
+      <c r="C63" s="5" t="s">
         <v>116</v>
       </c>
       <c r="D63" s="4" t="s">
@@ -8458,7 +8461,7 @@
       <c r="B64" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="C64" s="5" t="s">
         <v>117</v>
       </c>
       <c r="D64" s="4" t="s">
@@ -8578,7 +8581,7 @@
       <c r="B65" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C65" s="4" t="s">
+      <c r="C65" s="5" t="s">
         <v>118</v>
       </c>
       <c r="D65" s="4" t="s">
@@ -8698,7 +8701,7 @@
       <c r="B66" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C66" s="4" t="s">
+      <c r="C66" s="5" t="s">
         <v>119</v>
       </c>
       <c r="D66" s="4" t="s">
@@ -8818,7 +8821,7 @@
       <c r="B67" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C67" s="4" t="s">
+      <c r="C67" s="5" t="s">
         <v>120</v>
       </c>
       <c r="D67" s="4" t="s">
@@ -8938,7 +8941,7 @@
       <c r="B68" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="5" t="s">
         <v>121</v>
       </c>
       <c r="D68" s="4" t="s">
@@ -9058,7 +9061,7 @@
       <c r="B69" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C69" s="4" t="s">
+      <c r="C69" s="5" t="s">
         <v>122</v>
       </c>
       <c r="D69" s="4" t="s">
@@ -9178,7 +9181,7 @@
       <c r="B70" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C70" s="4" t="s">
+      <c r="C70" s="5" t="s">
         <v>123</v>
       </c>
       <c r="D70" s="4" t="s">
@@ -9298,7 +9301,7 @@
       <c r="B71" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C71" s="4" t="s">
+      <c r="C71" s="5" t="s">
         <v>124</v>
       </c>
       <c r="D71" s="4" t="s">
@@ -9418,7 +9421,7 @@
       <c r="B72" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="C72" s="5" t="s">
         <v>126</v>
       </c>
       <c r="D72" s="4" t="s">
@@ -9538,7 +9541,7 @@
       <c r="B73" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C73" s="4" t="s">
+      <c r="C73" s="5" t="s">
         <v>127</v>
       </c>
       <c r="D73" s="4" t="s">
@@ -9658,7 +9661,7 @@
       <c r="B74" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C74" s="4" t="s">
+      <c r="C74" s="5" t="s">
         <v>128</v>
       </c>
       <c r="D74" s="4" t="s">
@@ -9778,7 +9781,7 @@
       <c r="B75" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="C75" s="5" t="s">
         <v>129</v>
       </c>
       <c r="D75" s="4" t="s">
@@ -9898,7 +9901,7 @@
       <c r="B76" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="C76" s="5" t="s">
         <v>130</v>
       </c>
       <c r="D76" s="4" t="s">
@@ -10018,7 +10021,7 @@
       <c r="B77" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C77" s="5" t="s">
         <v>131</v>
       </c>
       <c r="D77" s="4" t="s">
@@ -10138,7 +10141,7 @@
       <c r="B78" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C78" s="5" t="s">
         <v>132</v>
       </c>
       <c r="D78" s="4" t="s">
@@ -10258,7 +10261,7 @@
       <c r="B79" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="C79" s="5" t="s">
         <v>134</v>
       </c>
       <c r="D79" s="4" t="s">
@@ -10378,7 +10381,7 @@
       <c r="B80" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C80" s="4" t="s">
+      <c r="C80" s="5" t="s">
         <v>136</v>
       </c>
       <c r="D80" s="4" t="s">
@@ -10498,7 +10501,7 @@
       <c r="B81" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="5" t="s">
         <v>137</v>
       </c>
       <c r="D81" s="4" t="s">
@@ -10618,7 +10621,7 @@
       <c r="B82" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="C82" s="5" t="s">
         <v>138</v>
       </c>
       <c r="D82" s="4" t="s">
@@ -10738,7 +10741,7 @@
       <c r="B83" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C83" s="4" t="s">
+      <c r="C83" s="5" t="s">
         <v>139</v>
       </c>
       <c r="D83" s="4" t="s">
@@ -10858,7 +10861,7 @@
       <c r="B84" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="5" t="s">
         <v>140</v>
       </c>
       <c r="D84" s="4" t="s">
@@ -10978,7 +10981,7 @@
       <c r="B85" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C85" s="4" t="s">
+      <c r="C85" s="5" t="s">
         <v>142</v>
       </c>
       <c r="D85" s="4" t="s">
@@ -11098,7 +11101,7 @@
       <c r="B86" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C86" s="4" t="s">
+      <c r="C86" s="5" t="s">
         <v>143</v>
       </c>
       <c r="D86" s="4" t="s">
@@ -11218,7 +11221,7 @@
       <c r="B87" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C87" s="4" t="s">
+      <c r="C87" s="5" t="s">
         <v>144</v>
       </c>
       <c r="D87" s="4" t="s">
@@ -11338,7 +11341,7 @@
       <c r="B88" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C88" s="4" t="s">
+      <c r="C88" s="5" t="s">
         <v>145</v>
       </c>
       <c r="D88" s="4" t="s">
@@ -11458,7 +11461,7 @@
       <c r="B89" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="C89" s="5" t="s">
         <v>146</v>
       </c>
       <c r="D89" s="4" t="s">
@@ -11578,7 +11581,7 @@
       <c r="B90" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C90" s="4" t="s">
+      <c r="C90" s="5" t="s">
         <v>147</v>
       </c>
       <c r="D90" s="4" t="s">
@@ -11698,7 +11701,7 @@
       <c r="B91" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C91" s="4" t="s">
+      <c r="C91" s="5" t="s">
         <v>148</v>
       </c>
       <c r="D91" s="4" t="s">
@@ -11818,7 +11821,7 @@
       <c r="B92" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C92" s="4" t="s">
+      <c r="C92" s="5" t="s">
         <v>149</v>
       </c>
       <c r="D92" s="4" t="s">
@@ -11938,7 +11941,7 @@
       <c r="B93" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C93" s="4" t="s">
+      <c r="C93" s="5" t="s">
         <v>150</v>
       </c>
       <c r="D93" s="4" t="s">
@@ -12058,7 +12061,7 @@
       <c r="B94" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C94" s="4" t="s">
+      <c r="C94" s="5" t="s">
         <v>151</v>
       </c>
       <c r="D94" s="4" t="s">
@@ -12178,7 +12181,7 @@
       <c r="B95" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C95" s="4" t="s">
+      <c r="C95" s="5" t="s">
         <v>152</v>
       </c>
       <c r="D95" s="4" t="s">
@@ -12298,7 +12301,7 @@
       <c r="B96" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C96" s="4" t="s">
+      <c r="C96" s="5" t="s">
         <v>153</v>
       </c>
       <c r="D96" s="4" t="s">
@@ -12418,7 +12421,7 @@
       <c r="B97" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C97" s="4" t="s">
+      <c r="C97" s="5" t="s">
         <v>154</v>
       </c>
       <c r="D97" s="4" t="s">
@@ -12538,7 +12541,7 @@
       <c r="B98" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C98" s="4" t="s">
+      <c r="C98" s="5" t="s">
         <v>155</v>
       </c>
       <c r="D98" s="4" t="s">
@@ -12658,7 +12661,7 @@
       <c r="B99" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C99" s="4" t="s">
+      <c r="C99" s="5" t="s">
         <v>156</v>
       </c>
       <c r="D99" s="4" t="s">
@@ -12778,7 +12781,7 @@
       <c r="B100" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C100" s="4" t="s">
+      <c r="C100" s="5" t="s">
         <v>157</v>
       </c>
       <c r="D100" s="4" t="s">
@@ -12898,7 +12901,7 @@
       <c r="B101" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C101" s="4" t="s">
+      <c r="C101" s="5" t="s">
         <v>158</v>
       </c>
       <c r="D101" s="4" t="s">
@@ -13018,7 +13021,7 @@
       <c r="B102" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C102" s="4" t="s">
+      <c r="C102" s="5" t="s">
         <v>159</v>
       </c>
       <c r="D102" s="4" t="s">
@@ -13138,7 +13141,7 @@
       <c r="B103" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C103" s="5" t="s">
         <v>160</v>
       </c>
       <c r="D103" s="4" t="s">

</xml_diff>